<commit_message>
Feat: Ajustes na lógica de matching
</commit_message>
<xml_diff>
--- a/inputs/De_Para_campos_gerenciais_EBTA.xlsx
+++ b/inputs/De_Para_campos_gerenciais_EBTA.xlsx
@@ -1434,11 +1434,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="51d5f85a-ee47-47b0-88a1-b6fc24e2aeee" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1669,27 +1670,17 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="51d5f85a-ee47-47b0-88a1-b6fc24e2aeee" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8A5F659-2FA3-4240-A4D6-27F34D90CCE2}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8D54FDD6-A2DA-4BE5-AD41-FE98702F0365}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="51d5f85a-ee47-47b0-88a1-b6fc24e2aeee"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="bad2e680-0a77-4f7e-94cc-de2e805fb83b"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1714,9 +1705,18 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8D54FDD6-A2DA-4BE5-AD41-FE98702F0365}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8A5F659-2FA3-4240-A4D6-27F34D90CCE2}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="51d5f85a-ee47-47b0-88a1-b6fc24e2aeee"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="bad2e680-0a77-4f7e-94cc-de2e805fb83b"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Feat: Ajuste de chave, validação de dados
</commit_message>
<xml_diff>
--- a/inputs/De_Para_campos_gerenciais_EBTA.xlsx
+++ b/inputs/De_Para_campos_gerenciais_EBTA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://flytour-my.sharepoint.com/personal/nicolas_cavalcante_flytour_com_br/Documents/Documentos/GitHub/projeto-conciliacao_ebta/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="8_{21FED629-1A5D-4403-97D4-F069104D19E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{14518FE2-314D-415C-8109-4A743D4074C1}"/>
+  <xr:revisionPtr revIDLastSave="26" documentId="8_{21FED629-1A5D-4403-97D4-F069104D19E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D2F9280-3A37-480B-BF96-43D153203FAE}"/>
   <bookViews>
     <workbookView xWindow="-21720" yWindow="1050" windowWidth="21840" windowHeight="13020" xr2:uid="{D02E9090-3899-4DD1-97E1-725276E51097}"/>
   </bookViews>
@@ -565,7 +565,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B50BFB2E-E356-4123-ACAF-01694ED01C70}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:F42"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -598,7 +597,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>4014606</v>
       </c>
@@ -618,7 +617,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>4275284</v>
       </c>
@@ -638,7 +637,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>2686650</v>
       </c>
@@ -658,7 +657,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>2893927</v>
       </c>
@@ -698,7 +697,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>3823642</v>
       </c>
@@ -718,7 +717,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="3">
         <v>3823646</v>
       </c>
@@ -738,7 +737,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>3823678</v>
       </c>
@@ -758,7 +757,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>3823684</v>
       </c>
@@ -778,7 +777,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>3825184</v>
       </c>
@@ -798,7 +797,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>3825184</v>
       </c>
@@ -818,7 +817,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>3825185</v>
       </c>
@@ -838,7 +837,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="4">
         <v>3825232</v>
       </c>
@@ -858,7 +857,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>3826373</v>
       </c>
@@ -878,7 +877,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
         <v>3826374</v>
       </c>
@@ -898,7 +897,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>4326326</v>
       </c>
@@ -918,7 +917,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>3826384</v>
       </c>
@@ -938,7 +937,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>3826383</v>
       </c>
@@ -958,7 +957,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>4513340</v>
       </c>
@@ -978,7 +977,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>3818353</v>
       </c>
@@ -1018,7 +1017,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="23" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>3816998</v>
       </c>
@@ -1038,7 +1037,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>2893927</v>
       </c>
@@ -1078,7 +1077,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="26" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
         <v>3823642</v>
       </c>
@@ -1098,7 +1097,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="27" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="3">
         <v>3823646</v>
       </c>
@@ -1118,7 +1117,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="28" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>3823678</v>
       </c>
@@ -1138,7 +1137,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="29" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>3823684</v>
       </c>
@@ -1158,7 +1157,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="30" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
         <v>3825184</v>
       </c>
@@ -1178,7 +1177,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>3825184</v>
       </c>
@@ -1198,7 +1197,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>3825185</v>
       </c>
@@ -1218,7 +1217,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="33" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="4">
         <v>3825232</v>
       </c>
@@ -1238,7 +1237,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="34" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="1">
         <v>3826373</v>
       </c>
@@ -1258,7 +1257,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="35" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="2">
         <v>3826374</v>
       </c>
@@ -1278,7 +1277,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="1">
         <v>4326326</v>
       </c>
@@ -1298,7 +1297,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="37" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="1">
         <v>3826384</v>
       </c>
@@ -1318,7 +1317,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="38" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="1">
         <v>3826383</v>
       </c>
@@ -1338,7 +1337,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="39" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="1">
         <v>4513340</v>
       </c>
@@ -1358,7 +1357,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="40" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="1">
         <v>3818353</v>
       </c>
@@ -1398,7 +1397,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="42" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" s="1">
         <v>3816998</v>
       </c>
@@ -1419,13 +1418,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F42" xr:uid="{B50BFB2E-E356-4123-ACAF-01694ED01C70}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="CNH INDUSTRIAL BRAS"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:F42" xr:uid="{B50BFB2E-E356-4123-ACAF-01694ED01C70}"/>
   <conditionalFormatting sqref="B1:B1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
@@ -1434,12 +1427,11 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="51d5f85a-ee47-47b0-88a1-b6fc24e2aeee" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1670,17 +1662,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="51d5f85a-ee47-47b0-88a1-b6fc24e2aeee" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8D54FDD6-A2DA-4BE5-AD41-FE98702F0365}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8A5F659-2FA3-4240-A4D6-27F34D90CCE2}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="51d5f85a-ee47-47b0-88a1-b6fc24e2aeee"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="bad2e680-0a77-4f7e-94cc-de2e805fb83b"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1705,18 +1707,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8A5F659-2FA3-4240-A4D6-27F34D90CCE2}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8D54FDD6-A2DA-4BE5-AD41-FE98702F0365}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="51d5f85a-ee47-47b0-88a1-b6fc24e2aeee"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="bad2e680-0a77-4f7e-94cc-de2e805fb83b"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Ajustes no corpo do email, e atualizações da interface
</commit_message>
<xml_diff>
--- a/inputs/De_Para_campos_gerenciais_EBTA.xlsx
+++ b/inputs/De_Para_campos_gerenciais_EBTA.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://flytour-my.sharepoint.com/personal/nicolas_cavalcante_flytour_com_br/Documents/Documentos/GitHub/projeto-conciliacao_ebta/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="8_{21FED629-1A5D-4403-97D4-F069104D19E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D2F9280-3A37-480B-BF96-43D153203FAE}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="8_{21FED629-1A5D-4403-97D4-F069104D19E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6DA5C4EC-F278-44DD-8F7A-854227B19F5C}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="1050" windowWidth="21840" windowHeight="13020" xr2:uid="{D02E9090-3899-4DD1-97E1-725276E51097}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D02E9090-3899-4DD1-97E1-725276E51097}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -565,6 +565,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B50BFB2E-E356-4123-ACAF-01694ED01C70}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:F42"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -597,7 +598,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>4014606</v>
       </c>
@@ -617,7 +618,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>4275284</v>
       </c>
@@ -637,7 +638,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>2686650</v>
       </c>
@@ -657,7 +658,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>2893927</v>
       </c>
@@ -697,7 +698,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>3823642</v>
       </c>
@@ -717,7 +718,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3">
         <v>3823646</v>
       </c>
@@ -737,7 +738,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>3823678</v>
       </c>
@@ -757,7 +758,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>3823684</v>
       </c>
@@ -777,7 +778,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>3825184</v>
       </c>
@@ -797,7 +798,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>3825184</v>
       </c>
@@ -817,7 +818,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>3825185</v>
       </c>
@@ -837,7 +838,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4">
         <v>3825232</v>
       </c>
@@ -857,7 +858,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>3826373</v>
       </c>
@@ -877,7 +878,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
         <v>3826374</v>
       </c>
@@ -897,7 +898,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>4326326</v>
       </c>
@@ -917,7 +918,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>3826384</v>
       </c>
@@ -937,7 +938,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>3826383</v>
       </c>
@@ -957,7 +958,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>4513340</v>
       </c>
@@ -977,7 +978,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>3818353</v>
       </c>
@@ -1017,7 +1018,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>3816998</v>
       </c>
@@ -1037,7 +1038,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>2893927</v>
       </c>
@@ -1077,7 +1078,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
         <v>3823642</v>
       </c>
@@ -1097,7 +1098,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="3">
         <v>3823646</v>
       </c>
@@ -1117,7 +1118,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>3823678</v>
       </c>
@@ -1137,7 +1138,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>3823684</v>
       </c>
@@ -1157,7 +1158,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
         <v>3825184</v>
       </c>
@@ -1177,7 +1178,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>3825184</v>
       </c>
@@ -1197,7 +1198,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>3825185</v>
       </c>
@@ -1217,7 +1218,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" s="4">
         <v>3825232</v>
       </c>
@@ -1237,7 +1238,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1">
         <v>3826373</v>
       </c>
@@ -1257,7 +1258,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" s="2">
         <v>3826374</v>
       </c>
@@ -1277,7 +1278,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1">
         <v>4326326</v>
       </c>
@@ -1297,7 +1298,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1">
         <v>3826384</v>
       </c>
@@ -1317,7 +1318,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1">
         <v>3826383</v>
       </c>
@@ -1337,7 +1338,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1">
         <v>4513340</v>
       </c>
@@ -1357,7 +1358,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1">
         <v>3818353</v>
       </c>
@@ -1397,7 +1398,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1">
         <v>3816998</v>
       </c>
@@ -1418,7 +1419,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F42" xr:uid="{B50BFB2E-E356-4123-ACAF-01694ED01C70}"/>
+  <autoFilter ref="A1:F42" xr:uid="{B50BFB2E-E356-4123-ACAF-01694ED01C70}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="CNH INDUSTRIAL BRAS"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <conditionalFormatting sqref="B1:B1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
@@ -1427,14 +1434,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="51d5f85a-ee47-47b0-88a1-b6fc24e2aeee" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101005A0345AEA7B61447A71507683AB7B56D" ma:contentTypeVersion="14" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="ee13b059e65c33a67f764d64691355ae">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="51d5f85a-ee47-47b0-88a1-b6fc24e2aeee" xmlns:ns4="bad2e680-0a77-4f7e-94cc-de2e805fb83b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7520885669c19df0b9cf18b53e58aa94" ns3:_="" ns4:_="">
     <xsd:import namespace="51d5f85a-ee47-47b0-88a1-b6fc24e2aeee"/>
@@ -1661,6 +1660,14 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="51d5f85a-ee47-47b0-88a1-b6fc24e2aeee" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1671,23 +1678,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8A5F659-2FA3-4240-A4D6-27F34D90CCE2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="51d5f85a-ee47-47b0-88a1-b6fc24e2aeee"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="bad2e680-0a77-4f7e-94cc-de2e805fb83b"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7DDE5FEC-F75B-48AF-A914-8B9DB50BB2C0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1706,6 +1696,23 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8A5F659-2FA3-4240-A4D6-27F34D90CCE2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="51d5f85a-ee47-47b0-88a1-b6fc24e2aeee"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="bad2e680-0a77-4f7e-94cc-de2e805fb83b"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8D54FDD6-A2DA-4BE5-AD41-FE98702F0365}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Feat: Alterações no arquivo final que sobe ao bradesco, alterações na interface e atualização de caminhos no executavel
</commit_message>
<xml_diff>
--- a/inputs/De_Para_campos_gerenciais_EBTA.xlsx
+++ b/inputs/De_Para_campos_gerenciais_EBTA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://flytour-my.sharepoint.com/personal/nicolas_cavalcante_flytour_com_br/Documents/Documentos/GitHub/projeto-conciliacao_ebta/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="8_{21FED629-1A5D-4403-97D4-F069104D19E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6DA5C4EC-F278-44DD-8F7A-854227B19F5C}"/>
+  <xr:revisionPtr revIDLastSave="37" documentId="8_{21FED629-1A5D-4403-97D4-F069104D19E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0FF4B666-1E00-47D9-A7D3-44BC86CB5A13}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D02E9090-3899-4DD1-97E1-725276E51097}"/>
   </bookViews>
@@ -56,9 +56,6 @@
     <t>Campo Produtividade</t>
   </si>
   <si>
-    <t>Hitachi Vantara</t>
-  </si>
-  <si>
     <t>Departamento</t>
   </si>
   <si>
@@ -68,9 +65,6 @@
     <t>Divisão</t>
   </si>
   <si>
-    <t>Bain Brasil</t>
-  </si>
-  <si>
     <t>Política</t>
   </si>
   <si>
@@ -150,6 +144,12 @@
   </si>
   <si>
     <t>Nome do Campo</t>
+  </si>
+  <si>
+    <t>HITACHI VANTARA ADMINISTRACAO DE DA</t>
+  </si>
+  <si>
+    <t>BAIN BRASIL</t>
   </si>
 </sst>
 </file>
@@ -589,7 +589,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>3</v>
@@ -598,24 +598,24 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>4014606</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -623,19 +623,19 @@
         <v>4275284</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -643,19 +643,19 @@
         <v>2686650</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="E4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -663,39 +663,39 @@
         <v>2893927</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>3816999</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -703,39 +703,39 @@
         <v>3823642</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="3">
+      <c r="A8" s="1">
         <v>3823646</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>22</v>
+      <c r="B8" s="1" t="s">
+        <v>20</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -743,19 +743,19 @@
         <v>3823678</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -763,19 +763,19 @@
         <v>3823684</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -783,19 +783,19 @@
         <v>3825184</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -803,19 +803,19 @@
         <v>3825184</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -823,19 +823,19 @@
         <v>3825185</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -843,19 +843,19 @@
         <v>3825232</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -863,19 +863,19 @@
         <v>3826373</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -883,19 +883,19 @@
         <v>3826374</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -903,19 +903,19 @@
         <v>4326326</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -923,19 +923,19 @@
         <v>3826384</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -943,19 +943,19 @@
         <v>3826383</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -963,19 +963,19 @@
         <v>4513340</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -983,39 +983,39 @@
         <v>3818353</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>3816999</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="23" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -1023,19 +1023,19 @@
         <v>3816998</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -1043,39 +1043,39 @@
         <v>2893927</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>3816999</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="26" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -1083,19 +1083,19 @@
         <v>3823642</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="27" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -1103,19 +1103,19 @@
         <v>3823646</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -1123,19 +1123,19 @@
         <v>3823678</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="29" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -1143,19 +1143,19 @@
         <v>3823684</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="30" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -1163,19 +1163,19 @@
         <v>3825184</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -1183,19 +1183,19 @@
         <v>3825184</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -1203,19 +1203,19 @@
         <v>3825185</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="33" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -1223,19 +1223,19 @@
         <v>3825232</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="34" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -1243,19 +1243,19 @@
         <v>3826373</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="35" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -1263,19 +1263,19 @@
         <v>3826374</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -1283,19 +1283,19 @@
         <v>4326326</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="37" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -1303,19 +1303,19 @@
         <v>3826384</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="38" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -1323,19 +1323,19 @@
         <v>3826383</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="39" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -1343,19 +1343,19 @@
         <v>4513340</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="40" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -1363,39 +1363,39 @@
         <v>3818353</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1">
         <v>3816999</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="42" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -1403,30 +1403,30 @@
         <v>3816998</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:F42" xr:uid="{B50BFB2E-E356-4123-ACAF-01694ED01C70}">
     <filterColumn colId="1">
       <filters>
-        <filter val="CNH INDUSTRIAL BRAS"/>
+        <filter val="HITACHI VANTARA ADMINISTRACAO DE DA"/>
       </filters>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="B1:B1048576">
+  <conditionalFormatting sqref="B1:B7 B10:B1048576 A8:B9">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
Feat: Inclusão de novas documentações no projeto, além de ajuste em tela_processamento, criando uma nova função baixar_canvas que força o uso da imagem fundo_fly durante o processamento
</commit_message>
<xml_diff>
--- a/inputs/De_Para_campos_gerenciais_EBTA.xlsx
+++ b/inputs/De_Para_campos_gerenciais_EBTA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://flytour-my.sharepoint.com/personal/nicolas_cavalcante_flytour_com_br/Documents/Documentos/GitHub/projeto-conciliacao_ebta/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="37" documentId="8_{21FED629-1A5D-4403-97D4-F069104D19E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0FF4B666-1E00-47D9-A7D3-44BC86CB5A13}"/>
+  <xr:revisionPtr revIDLastSave="38" documentId="8_{21FED629-1A5D-4403-97D4-F069104D19E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4C3962E6-A6F9-4085-A160-C66FFF056FC3}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D02E9090-3899-4DD1-97E1-725276E51097}"/>
   </bookViews>
@@ -565,7 +565,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B50BFB2E-E356-4123-ACAF-01694ED01C70}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:F42"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -618,7 +617,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>4275284</v>
       </c>
@@ -638,7 +637,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>2686650</v>
       </c>
@@ -658,7 +657,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>2893927</v>
       </c>
@@ -678,7 +677,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>3816999</v>
       </c>
@@ -698,7 +697,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>3823642</v>
       </c>
@@ -718,7 +717,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>3823646</v>
       </c>
@@ -738,7 +737,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>3823678</v>
       </c>
@@ -758,7 +757,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>3823684</v>
       </c>
@@ -778,7 +777,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>3825184</v>
       </c>
@@ -798,7 +797,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>3825184</v>
       </c>
@@ -818,7 +817,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>3825185</v>
       </c>
@@ -838,7 +837,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="4">
         <v>3825232</v>
       </c>
@@ -858,7 +857,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>3826373</v>
       </c>
@@ -878,7 +877,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
         <v>3826374</v>
       </c>
@@ -898,7 +897,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>4326326</v>
       </c>
@@ -918,7 +917,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>3826384</v>
       </c>
@@ -938,7 +937,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>3826383</v>
       </c>
@@ -958,7 +957,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>4513340</v>
       </c>
@@ -978,7 +977,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>3818353</v>
       </c>
@@ -998,7 +997,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>3816999</v>
       </c>
@@ -1018,7 +1017,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="23" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>3816998</v>
       </c>
@@ -1038,7 +1037,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>2893927</v>
       </c>
@@ -1058,7 +1057,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="25" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>3816999</v>
       </c>
@@ -1078,7 +1077,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
         <v>3823642</v>
       </c>
@@ -1098,7 +1097,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="27" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="3">
         <v>3823646</v>
       </c>
@@ -1118,7 +1117,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="28" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>3823678</v>
       </c>
@@ -1138,7 +1137,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="29" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>3823684</v>
       </c>
@@ -1158,7 +1157,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="30" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
         <v>3825184</v>
       </c>
@@ -1178,7 +1177,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>3825184</v>
       </c>
@@ -1198,7 +1197,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>3825185</v>
       </c>
@@ -1218,7 +1217,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="33" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="4">
         <v>3825232</v>
       </c>
@@ -1238,7 +1237,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="34" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="1">
         <v>3826373</v>
       </c>
@@ -1258,7 +1257,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="35" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="2">
         <v>3826374</v>
       </c>
@@ -1278,7 +1277,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="1">
         <v>4326326</v>
       </c>
@@ -1298,7 +1297,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="37" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="1">
         <v>3826384</v>
       </c>
@@ -1318,7 +1317,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="38" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="1">
         <v>3826383</v>
       </c>
@@ -1338,7 +1337,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="39" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="1">
         <v>4513340</v>
       </c>
@@ -1358,7 +1357,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="40" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="1">
         <v>3818353</v>
       </c>
@@ -1378,7 +1377,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="41" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="1">
         <v>3816999</v>
       </c>
@@ -1398,7 +1397,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="42" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" s="1">
         <v>3816998</v>
       </c>
@@ -1419,13 +1418,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F42" xr:uid="{B50BFB2E-E356-4123-ACAF-01694ED01C70}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="HITACHI VANTARA ADMINISTRACAO DE DA"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
   <conditionalFormatting sqref="B1:B7 B10:B1048576 A8:B9">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
@@ -1434,6 +1426,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="51d5f85a-ee47-47b0-88a1-b6fc24e2aeee" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101005A0345AEA7B61447A71507683AB7B56D" ma:contentTypeVersion="14" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="ee13b059e65c33a67f764d64691355ae">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="51d5f85a-ee47-47b0-88a1-b6fc24e2aeee" xmlns:ns4="bad2e680-0a77-4f7e-94cc-de2e805fb83b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7520885669c19df0b9cf18b53e58aa94" ns3:_="" ns4:_="">
     <xsd:import namespace="51d5f85a-ee47-47b0-88a1-b6fc24e2aeee"/>
@@ -1660,14 +1660,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="51d5f85a-ee47-47b0-88a1-b6fc24e2aeee" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1678,6 +1670,23 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8A5F659-2FA3-4240-A4D6-27F34D90CCE2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="51d5f85a-ee47-47b0-88a1-b6fc24e2aeee"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="bad2e680-0a77-4f7e-94cc-de2e805fb83b"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7DDE5FEC-F75B-48AF-A914-8B9DB50BB2C0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1696,23 +1705,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8A5F659-2FA3-4240-A4D6-27F34D90CCE2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="51d5f85a-ee47-47b0-88a1-b6fc24e2aeee"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="bad2e680-0a77-4f7e-94cc-de2e805fb83b"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8D54FDD6-A2DA-4BE5-AD41-FE98702F0365}">
   <ds:schemaRefs>

</xml_diff>